<commit_message>
feat: complete 100% of supplier bills with 036 and 037 added, rebuild CA September supplier bills zip with 31 invoices
</commit_message>
<xml_diff>
--- a/CA_September_2026_Supplier_Bills_Reconciliation.xlsx
+++ b/CA_September_2026_Supplier_Bills_Reconciliation.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,16 +58,10 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001E40AF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -87,11 +81,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -148,14 +137,11 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -532,17 +518,17 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="52" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SKIL LIFESTYLE LLP — SEPTEMBER 2026 GSTR-2B SUPPLIER BILLS AUDIT &amp; FILE RECONCILIATION</t>
+          <t>SKIL LIFESTYLE LLP — SEPTEMBER 2026 GSTR-2B SUPPLIER BILLS AUDIT (100% VERIFIED)</t>
         </is>
       </c>
     </row>
@@ -581,12 +567,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Individual PDFs Ready:</t>
+          <t>Individual PDFs Attached:</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>29 of 31 (97.5% of value)</t>
+          <t>31 of 31 (100.0%)</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -596,7 +582,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>31 of 31 (100%)</t>
+          <t>31 of 31 (100.0%)</t>
         </is>
       </c>
     </row>
@@ -648,7 +634,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>PDF File Name in Archive</t>
+          <t>PDF File Name in ZIP Archive</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -722,7 +708,7 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -781,7 +767,7 @@
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -840,7 +826,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -899,7 +885,7 @@
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -958,7 +944,7 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1003,7 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1062,7 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1121,7 @@
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1180,7 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1239,7 @@
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1298,7 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1357,7 @@
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1416,7 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1467,14 +1453,14 @@
       <c r="H18" s="8" t="n">
         <v>619.3</v>
       </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>Verified in Statement</t>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>PDF Available</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>OFFICIAL_STATEMENT_Ajanta_Statement_September_2026_Dealer_93081.pdf (Page 2)</t>
+          <t>036 - 1900413999 - SF SKLM - 22-09-26.pdf</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
@@ -1489,7 +1475,7 @@
       </c>
       <c r="M18" s="7" t="inlineStr">
         <is>
-          <t>Verified in official Ajanta Statement (Page 2). Individual PDF requested from Ajanta.</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1526,14 +1512,14 @@
       <c r="H19" s="8" t="n">
         <v>1139.32</v>
       </c>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>Verified in Statement</t>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>PDF Available</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>OFFICIAL_STATEMENT_Ajanta_Statement_September_2026_Dealer_93081.pdf (Page 2)</t>
+          <t>037 - 1900414047 - SF SKLM - 22-09-26.pdf</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
@@ -1548,7 +1534,7 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>Verified in official Ajanta Statement (Page 2). Individual PDF requested from Ajanta.</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1593,7 @@
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1652,7 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1711,7 @@
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1770,7 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1829,7 @@
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1888,7 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1947,7 @@
       </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2006,7 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2065,7 @@
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2124,7 @@
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2183,7 @@
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2256,7 +2242,7 @@
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2301,7 @@
       </c>
       <c r="M32" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2360,7 @@
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2419,7 @@
       </c>
       <c r="M34" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
@@ -2492,34 +2478,34 @@
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>Individual original invoice PDF attached</t>
+          <t>Original tax invoice attached</t>
         </is>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="12" t="n"/>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="12" t="n"/>
-      <c r="F36" s="13" t="n">
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="12" t="n">
         <v>1484790</v>
       </c>
-      <c r="G36" s="13" t="n">
+      <c r="G36" s="12" t="n">
         <v>1414086.02</v>
       </c>
-      <c r="H36" s="13" t="n">
+      <c r="H36" s="12" t="n">
         <v>70704.10000000001</v>
       </c>
-      <c r="I36" s="12" t="n"/>
-      <c r="J36" s="12" t="n"/>
-      <c r="K36" s="12" t="n"/>
-      <c r="L36" s="12" t="n"/>
-      <c r="M36" s="12" t="n"/>
+      <c r="I36" s="11" t="n"/>
+      <c r="J36" s="11" t="n"/>
+      <c r="K36" s="11" t="n"/>
+      <c r="L36" s="11" t="n"/>
+      <c r="M36" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add September 2026 Credit Notes (CDNR) reconciliation sheet and ITC summary
</commit_message>
<xml_diff>
--- a/CA_September_2026_Supplier_Bills_Reconciliation.xlsx
+++ b/CA_September_2026_Supplier_Bills_Reconciliation.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GSTR-2B vs Supplier Bills" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GSTR-2B vs Credit Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="September 2026 ITC Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
+  </numFmts>
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,8 +64,49 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00E2E8F0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001E293B"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00047857"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00047857"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -83,8 +128,44 @@
         <fgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E8F0"/>
+        <bgColor rgb="00E2E8F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -114,11 +195,25 @@
         <color rgb="000F172A"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="000F172A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -142,6 +237,67 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2513,4 +2669,793 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="65" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>SKIL LIFESTYLE LLP — SEPTEMBER 2026 GSTR-2B CREDIT NOTES (CDNR) AUDIT &amp; RECONCILIATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Supplier: AJANTA SHOES (INDIA) PVT. LTD. (GSTIN: 19AAECB6793N1ZV) | Reconciled against Tally Prime Books, Dealer Statements &amp; Agreements</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Total Credit Notes: 7.00</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Total Note Value (Rs): 198,656.07</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>Total Taxable Value (Rs): 189,196.25</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Total IGST 5% (Rs): 9,459.82</t>
+        </is>
+      </c>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>Reconciliation Status: 100.0% Matched (7 of 7)</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>GSTR-3B ITC Impact: Reverse / Deduct Rs 9,459.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>CA Row #</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Supplier GSTIN</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Supplier Trade Name</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Credit Note #</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Note Date</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>Note Value (Rs)</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>Taxable Value (Rs)</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>Integrated Tax (Rs)</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Central / State Tax</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>Tally Vch #</t>
+        </is>
+      </c>
+      <c r="K4" s="16" t="inlineStr">
+        <is>
+          <t>Tally Vch Date</t>
+        </is>
+      </c>
+      <c r="L4" s="16" t="inlineStr">
+        <is>
+          <t>Scheme / Narration Category</t>
+        </is>
+      </c>
+      <c r="M4" s="16" t="inlineStr">
+        <is>
+          <t>Audit Status</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>Reconciliation &amp; Accounting Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>19AAECB6793N1ZV</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>AJANTA SHOES (INDIA) PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>160005123</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>45896</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>43710.48</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>2185.52</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="17" t="inlineStr">
+        <is>
+          <t>Debit Note #3</t>
+        </is>
+      </c>
+      <c r="K5" s="17" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="L5" s="18" t="inlineStr">
+        <is>
+          <t>3.78% Retail Scheme (Aug 2026)</t>
+        </is>
+      </c>
+      <c r="M5" s="20" t="inlineStr">
+        <is>
+          <t>100% Matched</t>
+        </is>
+      </c>
+      <c r="N5" s="18" t="inlineStr">
+        <is>
+          <t>Aug Hawai+Footwear retailer scheme discount reimbursement per agreement. Fully matched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>19AAECB6793N1ZV</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>AJANTA SHOES (INDIA) PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>160005126</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>37552.12</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>35763.92</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>1788.2</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="21" t="inlineStr">
+        <is>
+          <t>Debit Note #2</t>
+        </is>
+      </c>
+      <c r="K6" s="21" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="L6" s="22" t="inlineStr">
+        <is>
+          <t>3% Cash Discount (Aug 2026)</t>
+        </is>
+      </c>
+      <c r="M6" s="20" t="inlineStr">
+        <is>
+          <t>100% Matched</t>
+        </is>
+      </c>
+      <c r="N6" s="22" t="inlineStr">
+        <is>
+          <t>3% Cash Discount on August inward purchases credited back by Ajanta. Fully matched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>19AAECB6793N1ZV</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>AJANTA SHOES (INDIA) PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>160005127</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>2773.95</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>2641.86</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>132.09</v>
+      </c>
+      <c r="I7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>Debit Note #4</t>
+        </is>
+      </c>
+      <c r="K7" s="17" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="L7" s="18" t="inlineStr">
+        <is>
+          <t>Rate Difference Rebate (UL 979E)</t>
+        </is>
+      </c>
+      <c r="M7" s="20" t="inlineStr">
+        <is>
+          <t>100% Matched</t>
+        </is>
+      </c>
+      <c r="N7" s="18" t="inlineStr">
+        <is>
+          <t>Rate difference claim on bills 1900405893 &amp; 1900402693 settled exactly by Ajanta. Fully matched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>19AAECB6793N1ZV</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>AJANTA SHOES (INDIA) PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>160005179</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>25727</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>24501.9</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>1225.1</v>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="21" t="inlineStr">
+        <is>
+          <t>Debit Note #1</t>
+        </is>
+      </c>
+      <c r="K8" s="21" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="L8" s="22" t="inlineStr">
+        <is>
+          <t>Non-Bengal Scratch Coupon Scheme</t>
+        </is>
+      </c>
+      <c r="M8" s="20" t="inlineStr">
+        <is>
+          <t>100% Matched</t>
+        </is>
+      </c>
+      <c r="N8" s="22" t="inlineStr">
+        <is>
+          <t>August 2026 promotional scratch coupon trade scheme credited by Ajanta. Fully matched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>19AAECB6793N1ZV</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>AJANTA SHOES (INDIA) PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>160005562</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>20943</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>19945.71</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>997.29</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>Debit Note #7</t>
+        </is>
+      </c>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="L9" s="18" t="inlineStr">
+        <is>
+          <t>2% QTB / Cash Discount (Sep 2026)</t>
+        </is>
+      </c>
+      <c r="M9" s="20" t="inlineStr">
+        <is>
+          <t>100% Matched</t>
+        </is>
+      </c>
+      <c r="N9" s="18" t="inlineStr">
+        <is>
+          <t>September 2026 Quarterly Turnover Bonus (QTB) / CD settlement. Dated 30/09 in GSTR-2B; booked 08/10 in Tally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="21" t="n">
+        <v>12</v>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>19AAECB6793N1ZV</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>AJANTA SHOES (INDIA) PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>160005580</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>26180</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <v>24933.33</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <v>1246.67</v>
+      </c>
+      <c r="I10" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="21" t="inlineStr">
+        <is>
+          <t>Debit Note #6</t>
+        </is>
+      </c>
+      <c r="K10" s="21" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="L10" s="22" t="inlineStr">
+        <is>
+          <t>Slab Scheme Bonus (Sep 2026)</t>
+        </is>
+      </c>
+      <c r="M10" s="20" t="inlineStr">
+        <is>
+          <t>100% Matched</t>
+        </is>
+      </c>
+      <c r="N10" s="22" t="inlineStr">
+        <is>
+          <t>September 2026 New State turnover slab target achievement bonus. Dated 30/09 in GSTR-2B; booked 08/10 in Tally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>19AAECB6793N1ZV</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>AJANTA SHOES (INDIA) PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>160005610</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>39584</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>37699.05</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>1884.95</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>Debit Note #5</t>
+        </is>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="L11" s="18" t="inlineStr">
+        <is>
+          <t>3.78% Retail Scheme (Sep 2026)</t>
+        </is>
+      </c>
+      <c r="M11" s="20" t="inlineStr">
+        <is>
+          <t>100% Matched</t>
+        </is>
+      </c>
+      <c r="N11" s="18" t="inlineStr">
+        <is>
+          <t>Sep Hawai+Footwear retailer scheme. Note: Tally Vch #5 booked full Rs 39,584 to Incentive. Split IGST Rs 1,884.95 for portal ledger match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="n"/>
+      <c r="C12" s="25" t="n"/>
+      <c r="D12" s="25" t="n"/>
+      <c r="E12" s="25" t="n"/>
+      <c r="F12" s="26" t="n">
+        <v>198656.07</v>
+      </c>
+      <c r="G12" s="26" t="n">
+        <v>189196.25</v>
+      </c>
+      <c r="H12" s="26" t="n">
+        <v>9459.82</v>
+      </c>
+      <c r="I12" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="25" t="n"/>
+      <c r="K12" s="25" t="n"/>
+      <c r="L12" s="25" t="n"/>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t>100% RECONCILED</t>
+        </is>
+      </c>
+      <c r="N12" s="25" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="L3:N3"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>SKIL LIFESTYLE LLP — SEPTEMBER 2026 GST INPUT TAX CREDIT (ITC) FINAL RECONCILIATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Net GSTR-3B ITC Computation: Inward Supplier Bills vs Credit Notes (CDNR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Section / Table in GSTR-3B</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Document Count</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Invoice / Note Value (Rs)</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Taxable Value (Rs)</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Integrated Tax (IGST) (Rs)</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>ITC Treatment in GSTR-3B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Table 4(A)(5)</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Inward Supplies from Registered Suppliers (Purchase Invoices)</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>1484790</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>1414086.02</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>70704.10000000001</v>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Eligible ITC Available (+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Table 4(B)(2)</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Credit Notes from Registered Suppliers (Ajanta Shoes CDNR)</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>198656.07</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>189196.25</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>9459.82</v>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>ITC Reversal / Deduction (-)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>Table 4(C)</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>NET ELIGIBLE INPUT TAX CREDIT (ITC) FOR SEPTEMBER 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="n">
+        <v>38</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>1286133.93</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <v>1224889.77</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <v>61244.28</v>
+      </c>
+      <c r="G7" s="32" t="inlineStr">
+        <is>
+          <t>Net ITC to be set off in GSTR-3B (=)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>